<commit_message>
Table import: an empty Excel template in the campus sheet's style, with hours
The template is built by backend/scripts/make_campus_template.py, like the
campus data sheet of stage 1: a row of groups over the headers, lists for
the kind of place and the building's status, a colour per kind, grey on
the columns a kind does not use, an instructions sheet and an example on
a sheet of its own. The sheet to fill is empty.

The reader takes what that sheet allows: an empty short name is the
building of the row above, "no study places" adds the building only, a
status (active, new, under construction), and opening hours for Sunday
to Thursday and for Friday (HH:MM-HH:MM or closed; empty: the usual
hours), checked again on save. A test reads the template's headers and
lists against the reader, and a filled-in copy of it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBYsCxt5GrWc3JhqYiChAW
</commit_message>
<xml_diff>
--- a/frontend/public/templates/buildings.xlsx
+++ b/frontend/public/templates/buildings.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="בניינים ומקומות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="הוראות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="דוגמה" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,17 +29,55 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,17 +85,88 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00A9D08E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F4B183"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E89AB8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="008FD3D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00A6A6A6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -417,82 +528,406 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>הבניין</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>המקום</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+      <c r="H1" s="4" t="n"/>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>חוות מחשבים</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="n"/>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>שעות פתיחה</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="n"/>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>איך מגיעים</t>
+        </is>
+      </c>
+      <c r="N1" s="9" t="inlineStr">
+        <is>
+          <t>מיקום על המפה, לא חובה</t>
+        </is>
+      </c>
+      <c r="O1" s="10" t="n"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
           <t>שם קצר</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>שם הבניין</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>מספר קומות</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>מצב הבניין</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>סוג המקום</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>שם המקום</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>קומה</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>כמה אנשים</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>שורות</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>עמדות בשורה</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
+        <is>
+          <t>ימים א'-ה'</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>יום ו'</t>
+        </is>
+      </c>
+      <c r="M2" s="11" t="inlineStr">
+        <is>
+          <t>הערת מיקום</t>
+        </is>
+      </c>
+      <c r="N2" s="11" t="inlineStr">
         <is>
           <t>קו רוחב</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O2" s="11" t="inlineStr">
         <is>
           <t>קו אורך</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="I1:J1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E3:E302">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$E3="חדר לימוד קבוצתי"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>$E3="מתחם לימוד פתוח"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$E3="ספרייה"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="3">
+      <formula>$E3="חוות מחשבים"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I3:J302">
+    <cfRule type="expression" priority="2" dxfId="4" stopIfTrue="0">
+      <formula>$E3="חדר לימוד קבוצתי"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="4" stopIfTrue="0">
+      <formula>$E3="מתחם לימוד פתוח"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="4" stopIfTrue="0">
+      <formula>$E3="ספרייה"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H302">
+    <cfRule type="expression" priority="8" dxfId="4" stopIfTrue="0">
+      <formula>$E3="חוות מחשבים"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:M302">
+    <cfRule type="expression" priority="9" dxfId="4" stopIfTrue="0">
+      <formula>$E3="אין מקומות לימוד"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="E3:E302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא מוכר" error="בוחרים ערך מהרשימה." type="list">
+      <formula1>"חדר לימוד קבוצתי,מתחם לימוד פתוח,ספרייה,חוות מחשבים,אין מקומות לימוד"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D3:D302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא מוכר" error="בוחרים ערך מהרשימה." type="list">
+      <formula1>"פעיל,חדש,בבנייה"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="115" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>איך ממלאים</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>1. כל בניין הוא בלוק של שורות. בשורה הראשונה שלו כותבים שם קצר, שם, מספר קומות ומצב.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>2. כל מקום לימוד בבניין מקבל שורה משלו. בשורות שמתחת משאירים את פרטי הבניין ריקים, וזה אומר "אותו בניין כמו למעלה".</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>3. השם הקצר: אותיות באנגלית, ספרות ומקף, כמו M או EM. הוא מופיע בשמות המקומות ועל השלטים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>4. בעמודה "סוג המקום" בוחרים מהרשימה. העמודות שלא שייכות לסוג נצבעות באפור, ואותן משאירים ריקות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>5. בניין בלי מקומות לימוד: שורה אחת, ובסוג המקום בוחרים "אין מקומות לימוד". הוא יופיע על המפה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>6. קומה: הכניסה היא קומה 0, ומעליה 1, 2 וכן הלאה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>7. חוות מחשבים: שורות ועמדות בשורה. נוצרת עמדה לכל שורה ועמודה, ומהן מפת העמדות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>8. שעות פתיחה: למשל 07:00-20:00, או "סגור". ריק נותן את השעות הרגילות: א'-ה' 07:00-20:00, ו' 07:00-14:00. שבת סגורה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>9. מיקום על המפה לא חובה: אפשר לקבוע אותו אחר כך בדף הניהול, ב"מיקום בניינים".</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>10. כשמעלים, האתר מראה קודם מה נמצא בטבלה, ושורה עם בעיה מסומנת עם הסיבה. שום דבר לא נשמר עד שמאשרים.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>דוגמה ממולאת יש בגיליון "דוגמה". ממלאים את הגיליון "בניינים ומקומות", והוא היחיד שנקרא.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>שם קצר</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>שם הבניין</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>מספר קומות</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>מצב הבניין</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>סוג המקום</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>שם המקום</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>קומה</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>כמה אנשים</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>שורות</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>עמדות בשורה</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>ימים א'-ה'</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="inlineStr">
+        <is>
+          <t>יום ו'</t>
+        </is>
+      </c>
+      <c r="M1" s="14" t="inlineStr">
         <is>
           <t>הערת מיקום</t>
+        </is>
+      </c>
+      <c r="N1" s="14" t="inlineStr">
+        <is>
+          <t>קו רוחב</t>
+        </is>
+      </c>
+      <c r="O1" s="14" t="inlineStr">
+        <is>
+          <t>קו אורך</t>
         </is>
       </c>
     </row>
@@ -512,69 +947,76 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>פעיל</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>חוות מחשבים</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>M206</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>5</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>8</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>07:00-20:00</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>בקומה הראשונה, משמאל למעלית</t>
+          <t>07:00-14:00</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ליד המעלית</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>בניין ההנדסה</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>חדר לימוד קבוצתי</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>M310</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>6</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>סגור</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>NX</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>הספרייה</t>
+          <t>בניין חדש</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -582,65 +1024,13 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ספרייה</t>
+          <t>בבנייה</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>אולם קריאה</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>הספרייה</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>מתחם לימוד פתוח</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>מרפסת</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>בניין הסטודנטים</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
+          <t>אין מקומות לימוד</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>